<commit_message>
Update tax credit files for latest thinking on tax credit availability
</commit_message>
<xml_diff>
--- a/InputData/elec/BSfGBP/BAU Subsidy for Grid Battery Production.xlsx
+++ b/InputData/elec/BSfGBP/BAU Subsidy for Grid Battery Production.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\elec\BSfGBP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BSfGBP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE210D11-D507-4B7D-9682-9ED38CE981CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBE71D76-7912-4BEC-A1F3-57F92E3FE77D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="2" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -125,14 +125,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -449,17 +448,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF982137-6F01-4109-8226-D4C6F3731BA9}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="101.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -467,37 +466,37 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" s="2">
         <v>2022</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>0.75350342301658668</v>
       </c>
@@ -505,7 +504,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>0.73</v>
       </c>
@@ -513,7 +512,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>0.03</v>
       </c>
@@ -529,9 +528,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B33CFD9F-5CAA-490F-A0C6-0C0A5236B09C}">
   <dimension ref="B2:K3"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.75">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B2">
         <v>2023</v>
       </c>
@@ -563,7 +562,7 @@
         <v>2032</v>
       </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.75">
+    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B3">
         <v>1</v>
       </c>
@@ -606,202 +605,226 @@
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.54296875" style="4" customWidth="1"/>
-    <col min="2" max="16384" width="8.7265625" style="4"/>
+    <col min="1" max="1" width="24.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.75">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4">
+      <c r="B1">
         <v>2021</v>
       </c>
-      <c r="C1" s="4">
+      <c r="C1">
         <v>2022</v>
       </c>
-      <c r="D1" s="4">
+      <c r="D1">
         <v>2023</v>
       </c>
-      <c r="E1" s="4">
+      <c r="E1">
         <v>2024</v>
       </c>
-      <c r="F1" s="4">
+      <c r="F1">
         <v>2025</v>
       </c>
-      <c r="G1" s="4">
+      <c r="G1">
         <v>2026</v>
       </c>
-      <c r="H1" s="4">
+      <c r="H1">
         <v>2027</v>
       </c>
-      <c r="I1" s="4">
+      <c r="I1">
         <v>2028</v>
       </c>
-      <c r="J1" s="4">
+      <c r="J1">
         <v>2029</v>
       </c>
-      <c r="K1" s="4">
+      <c r="K1">
         <v>2030</v>
       </c>
-      <c r="L1" s="4">
+      <c r="L1">
         <v>2031</v>
       </c>
-      <c r="M1" s="4">
+      <c r="M1">
         <v>2032</v>
       </c>
-      <c r="N1" s="4">
+      <c r="N1">
         <v>2033</v>
       </c>
-      <c r="O1" s="4">
+      <c r="O1">
         <v>2034</v>
       </c>
-      <c r="P1" s="4">
+      <c r="P1">
         <v>2035</v>
       </c>
-      <c r="Q1" s="4">
+      <c r="Q1">
         <v>2036</v>
       </c>
-      <c r="R1" s="4">
+      <c r="R1">
         <v>2037</v>
       </c>
-      <c r="S1" s="4">
+      <c r="S1">
         <v>2038</v>
       </c>
-      <c r="T1" s="4">
+      <c r="T1">
         <v>2039</v>
       </c>
-      <c r="U1" s="4">
+      <c r="U1">
         <v>2040</v>
       </c>
-      <c r="V1" s="4">
+      <c r="V1">
         <v>2041</v>
       </c>
-      <c r="W1" s="4">
+      <c r="W1">
         <v>2042</v>
       </c>
-      <c r="X1" s="4">
+      <c r="X1">
         <v>2043</v>
       </c>
-      <c r="Y1" s="4">
+      <c r="Y1">
         <v>2044</v>
       </c>
-      <c r="Z1" s="4">
+      <c r="Z1">
         <v>2045</v>
       </c>
-      <c r="AA1" s="4">
+      <c r="AA1">
         <v>2046</v>
       </c>
-      <c r="AB1" s="4">
+      <c r="AB1">
         <v>2047</v>
       </c>
-      <c r="AC1" s="4">
+      <c r="AC1">
         <v>2048</v>
       </c>
-      <c r="AD1" s="4">
+      <c r="AD1">
         <v>2049</v>
       </c>
-      <c r="AE1" s="4">
+      <c r="AE1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.75">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4">
-        <v>0</v>
-      </c>
-      <c r="C2" s="4">
-        <v>0</v>
-      </c>
-      <c r="D2" s="4">
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
         <f>45*About!$A$12*10^3</f>
         <v>33907.654035746404</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2">
         <f>45*About!$A$13*10^3</f>
         <v>32850</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2">
         <f>$E2*(1-About!$A$14)^(F1-$E1)*'Phase Out'!D3</f>
         <v>31864.5</v>
       </c>
-      <c r="G2" s="4">
-        <v>0</v>
-      </c>
-      <c r="H2" s="4">
-        <v>0</v>
-      </c>
-      <c r="I2" s="4">
-        <v>0</v>
-      </c>
-      <c r="J2" s="4">
-        <v>0</v>
-      </c>
-      <c r="K2" s="4">
-        <v>0</v>
-      </c>
-      <c r="L2" s="4">
-        <v>0</v>
-      </c>
-      <c r="M2" s="4">
-        <v>0</v>
-      </c>
-      <c r="N2" s="4">
-        <v>0</v>
-      </c>
-      <c r="O2" s="4">
-        <v>0</v>
-      </c>
-      <c r="P2" s="4">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="4">
-        <v>0</v>
-      </c>
-      <c r="R2" s="4">
-        <v>0</v>
-      </c>
-      <c r="S2" s="4">
-        <v>0</v>
-      </c>
-      <c r="T2" s="4">
-        <v>0</v>
-      </c>
-      <c r="U2" s="4">
-        <v>0</v>
-      </c>
-      <c r="V2" s="4">
-        <v>0</v>
-      </c>
-      <c r="W2" s="4">
-        <v>0</v>
-      </c>
-      <c r="X2" s="4">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="4">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="4">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="4">
+      <c r="G2">
+        <f>$E2*(1-About!$A$14)^(G1-$E1)*'Phase Out'!E3</f>
+        <v>30908.564999999999</v>
+      </c>
+      <c r="H2">
+        <f>$E2*(1-About!$A$14)^(H1-$E1)*'Phase Out'!F3</f>
+        <v>29981.30805</v>
+      </c>
+      <c r="I2">
+        <f>$E2*(1-About!$A$14)^(I1-$E1)*'Phase Out'!G3</f>
+        <v>29081.868808499999</v>
+      </c>
+      <c r="J2">
+        <f>$E2*(1-About!$A$14)^(J1-$E1)*'Phase Out'!H3</f>
+        <v>28209.412744244997</v>
+      </c>
+      <c r="K2">
+        <f>$E2*(1-About!$A$14)^(K1-$E1)*'Phase Out'!I3</f>
+        <v>20522.347771438235</v>
+      </c>
+      <c r="L2">
+        <f>$E2*(1-About!$A$14)^(L1-$E1)*'Phase Out'!J3</f>
+        <v>13271.118225530059</v>
+      </c>
+      <c r="M2">
+        <f>$E2*(1-About!$A$14)^(M1-$E1)*'Phase Out'!K3</f>
+        <v>6436.4923393820782</v>
+      </c>
+      <c r="N2">
+        <f>$E2*(1-About!$A$14)^(N1-$E1)*'Phase Out'!L3</f>
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <f>$E2*(1-About!$A$14)^(O1-$E1)*'Phase Out'!M3</f>
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <f>$E2*(1-About!$A$14)^(P1-$E1)*'Phase Out'!N3</f>
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <f>$E2*(1-About!$A$14)^(Q1-$E1)*'Phase Out'!O3</f>
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <f>$E2*(1-About!$A$14)^(R1-$E1)*'Phase Out'!P3</f>
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <f>$E2*(1-About!$A$14)^(S1-$E1)*'Phase Out'!Q3</f>
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <f>$E2*(1-About!$A$14)^(T1-$E1)*'Phase Out'!R3</f>
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <f>$E2*(1-About!$A$14)^(U1-$E1)*'Phase Out'!S3</f>
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <f>$E2*(1-About!$A$14)^(V1-$E1)*'Phase Out'!T3</f>
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <f>$E2*(1-About!$A$14)^(W1-$E1)*'Phase Out'!U3</f>
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <f>$E2*(1-About!$A$14)^(X1-$E1)*'Phase Out'!V3</f>
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <f>$E2*(1-About!$A$14)^(Y1-$E1)*'Phase Out'!W3</f>
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <f>$E2*(1-About!$A$14)^(Z1-$E1)*'Phase Out'!X3</f>
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <f>$E2*(1-About!$A$14)^(AA1-$E1)*'Phase Out'!Y3</f>
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <f>$E2*(1-About!$A$14)^(AB1-$E1)*'Phase Out'!Z3</f>
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <f>$E2*(1-About!$A$14)^(AC1-$E1)*'Phase Out'!AA3</f>
+        <v>0</v>
+      </c>
+      <c r="AD2">
+        <f>$E2*(1-About!$A$14)^(AD1-$E1)*'Phase Out'!AB3</f>
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <f>$E2*(1-About!$A$14)^(AE1-$E1)*'Phase Out'!AC3</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>